<commit_message>
Replace Excel workbook (.xlsx) (binary change)
Replaced a binary Excel workbook (filename contains Japanese characters). Git shows the blob changed from fee56bb to 9536700; contents are binary so no text diff is available. This change only updates the .xlsx file; no source code was modified.
</commit_message>
<xml_diff>
--- a/配布データ一覧.xlsx
+++ b/配布データ一覧.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="27830"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30326"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\■■■■■■New＿滋賀医大\■■講義関連\京都府大\講義資料\2024_R\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\aharada\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{755E91ED-69D0-4BB2-8A27-B290D9163415}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AE83F87A-4D71-438F-A85C-F4E4AC8BB45F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="52717" yWindow="25" windowWidth="18031" windowHeight="12847" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="250" uniqueCount="175">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="245" uniqueCount="181">
   <si>
     <t>#02_0902</t>
     <phoneticPr fontId="1"/>
@@ -400,46 +400,6 @@
     <phoneticPr fontId="1"/>
   </si>
   <si>
-    <t>#1_保健統計学実習_0831.pdf</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>#1_保健統計学実習_0831_x4.pdf</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>#02_保健統計学実習_0901.pdf</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>#02_保健統計学実習_0901_x4.pdf</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>#03_保健統計学実習_0905.pdf</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>#03_保健統計学実習_0905_x4.pdf</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>#04_保健統計実習_0906.pdf</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>#04_保健統計実習_0906_x4.pdf</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>#5_保健統計学実習_0908.pdf</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>#5_保健統計学実習_0908_x4.pdf</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
     <t>lipid_Data.csv</t>
     <phoneticPr fontId="1"/>
   </si>
@@ -504,10 +464,6 @@
     <phoneticPr fontId="1"/>
   </si>
   <si>
-    <t>8_questionnaire</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
     <t>2way.csv</t>
     <phoneticPr fontId="1"/>
   </si>
@@ -568,27 +524,11 @@
     <phoneticPr fontId="1"/>
   </si>
   <si>
-    <t>TokyoSTAT_P25.csv</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>TokyoSTAT_P25.sav</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
     <t>Candy_cluster.csv</t>
     <phoneticPr fontId="1"/>
   </si>
   <si>
     <t>Candy_cluster.sav</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>beer_2.csv</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>beer_2.sav</t>
     <phoneticPr fontId="1"/>
   </si>
   <si>
@@ -650,36 +590,6 @@
     <t>Sleepdata(原本）.xlsx</t>
     <rPh sb="10" eb="12">
       <t>ゲンホン</t>
-    </rPh>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>2024_講義レジュメ.pdf</t>
-    <rPh sb="5" eb="7">
-      <t>コウギ</t>
-    </rPh>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>2024_本実習の課題.pdf</t>
-    <rPh sb="5" eb="8">
-      <t>ホンジッシュウ</t>
-    </rPh>
-    <rPh sb="9" eb="11">
-      <t>カダイ</t>
-    </rPh>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>作成した調査票のLINK情報,txt</t>
-    <rPh sb="0" eb="2">
-      <t>サクセイ</t>
-    </rPh>
-    <rPh sb="4" eb="7">
-      <t>チョウサヒョウ</t>
-    </rPh>
-    <rPh sb="12" eb="14">
-      <t>ジョウホウ</t>
     </rPh>
     <phoneticPr fontId="1"/>
   </si>
@@ -709,6 +619,108 @@
     <rPh sb="6" eb="12">
       <t>イガクトウケイニュウモン</t>
     </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>2026_講義レジュメ.pdf</t>
+    <rPh sb="5" eb="7">
+      <t>コウギ</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>#1_保健統計学実習_2026.pdf</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>#02_保健統計学実習_2026.pdf</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>#03_保健統計学実習_2026.pdf</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>#04_保健統計実習_2026.pdf</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>#5_DeepLearning_2026.pdfpdf</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>5_Rcode</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>7_questionnaire</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>6_python</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>#1_NCD_stat _ncd course.ipynb</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>#02_ttest_chi-square_NCD course</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>beer_2,csv</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>Candy_Bars.sav</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>mnist(1)</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>fashion_kadai</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>food_CNN_classification_学生版</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>food_CNN_classification_自己学習版</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>food_YOLO_exercise</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>8 他</t>
+    <rPh sb="2" eb="3">
+      <t>ホカ</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>Ann1.zip</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>Ann2.zip</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>Ann3.zip</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>Ann4.zip</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>学習済みモデル.txt</t>
     <phoneticPr fontId="1"/>
   </si>
 </sst>
@@ -792,7 +804,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -805,9 +817,6 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1">
       <alignment vertical="center"/>
     </xf>
@@ -816,6 +825,15 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
+      <alignment vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1098,19 +1116,19 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:G56"/>
-  <sheetFormatPr defaultColWidth="8.69921875" defaultRowHeight="13.5" customHeight="1" x14ac:dyDescent="0.45"/>
+  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="13.5" customHeight="1" x14ac:dyDescent="0.55000000000000004"/>
   <cols>
-    <col min="1" max="1" width="17.19921875" style="1" customWidth="1"/>
-    <col min="2" max="2" width="21.3984375" style="1" customWidth="1"/>
-    <col min="3" max="3" width="29.19921875" style="1" customWidth="1"/>
-    <col min="4" max="4" width="30.09765625" style="1" customWidth="1"/>
-    <col min="5" max="5" width="30.19921875" style="1" customWidth="1"/>
-    <col min="6" max="6" width="26.8984375" style="1" customWidth="1"/>
-    <col min="7" max="7" width="28.796875" style="1" customWidth="1"/>
-    <col min="8" max="16384" width="8.69921875" style="1"/>
+    <col min="1" max="1" width="17.1640625" style="1" customWidth="1"/>
+    <col min="2" max="2" width="21.4140625" style="1" customWidth="1"/>
+    <col min="3" max="3" width="29.1640625" style="1" customWidth="1"/>
+    <col min="4" max="4" width="30.08203125" style="1" customWidth="1"/>
+    <col min="5" max="5" width="30.1640625" style="1" customWidth="1"/>
+    <col min="6" max="6" width="26.9140625" style="1" customWidth="1"/>
+    <col min="7" max="7" width="28.83203125" style="1" customWidth="1"/>
+    <col min="8" max="16384" width="8.6640625" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" ht="31.95" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:7" ht="32" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A1" s="2"/>
       <c r="B1" s="2" t="s">
         <v>101</v>
@@ -1131,12 +1149,12 @@
         <v>103</v>
       </c>
     </row>
-    <row r="2" spans="1:7" ht="13.5" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="2" spans="1:7" ht="13.5" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="B2" s="1" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="3" spans="1:7" ht="13.5" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="3" spans="1:7" ht="13.5" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A3" s="1" t="s">
         <v>3</v>
       </c>
@@ -1156,7 +1174,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="4" spans="1:7" ht="13.5" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="4" spans="1:7" ht="13.5" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="C4" s="1" t="s">
         <v>5</v>
       </c>
@@ -1173,7 +1191,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="5" spans="1:7" ht="13.5" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="5" spans="1:7" ht="13.5" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A5" s="3"/>
       <c r="B5" s="3"/>
       <c r="C5" s="3"/>
@@ -1182,7 +1200,7 @@
       <c r="F5" s="3"/>
       <c r="G5" s="3"/>
     </row>
-    <row r="6" spans="1:7" ht="13.5" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="6" spans="1:7" ht="13.5" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A6" s="1" t="s">
         <v>6</v>
       </c>
@@ -1199,7 +1217,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="7" spans="1:7" ht="13.5" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="7" spans="1:7" ht="13.5" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A7" s="1" t="s">
         <v>11</v>
       </c>
@@ -1219,7 +1237,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="8" spans="1:7" ht="13.5" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="8" spans="1:7" ht="13.5" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="C8" s="1" t="s">
         <v>8</v>
       </c>
@@ -1233,7 +1251,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="9" spans="1:7" ht="13.5" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="9" spans="1:7" ht="13.5" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="D9" s="1" t="s">
         <v>30</v>
       </c>
@@ -1241,37 +1259,37 @@
         <v>61</v>
       </c>
     </row>
-    <row r="10" spans="1:7" ht="13.5" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="10" spans="1:7" ht="13.5" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="E10" s="1" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="11" spans="1:7" ht="13.5" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="11" spans="1:7" ht="13.5" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="E11" s="1" t="s">
         <v>55</v>
       </c>
     </row>
-    <row r="12" spans="1:7" ht="13.5" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="12" spans="1:7" ht="13.5" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="E12" s="1" t="s">
         <v>57</v>
       </c>
     </row>
-    <row r="13" spans="1:7" ht="13.5" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="13" spans="1:7" ht="13.5" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="E13" s="1" t="s">
         <v>59</v>
       </c>
     </row>
-    <row r="14" spans="1:7" ht="13.5" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="14" spans="1:7" ht="13.5" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="E14" s="1" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="15" spans="1:7" ht="13.5" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="15" spans="1:7" ht="13.5" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="E15" s="1" t="s">
         <v>53</v>
       </c>
     </row>
-    <row r="16" spans="1:7" ht="13.5" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="16" spans="1:7" ht="13.5" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A16" s="3"/>
       <c r="B16" s="3"/>
       <c r="C16" s="3"/>
@@ -1280,7 +1298,7 @@
       <c r="F16" s="3"/>
       <c r="G16" s="3"/>
     </row>
-    <row r="17" spans="1:7" ht="13.5" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="17" spans="1:7" ht="13.5" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A17" s="1" t="s">
         <v>12</v>
       </c>
@@ -1300,7 +1318,7 @@
         <v>95</v>
       </c>
     </row>
-    <row r="18" spans="1:7" ht="13.5" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="18" spans="1:7" ht="13.5" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="C18" s="1" t="s">
         <v>10</v>
       </c>
@@ -1317,7 +1335,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="19" spans="1:7" ht="13.5" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="19" spans="1:7" ht="13.5" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="D19" s="1" t="s">
         <v>33</v>
       </c>
@@ -1331,7 +1349,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="20" spans="1:7" ht="13.5" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="20" spans="1:7" ht="13.5" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="D20" s="1" t="s">
         <v>31</v>
       </c>
@@ -1342,7 +1360,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="21" spans="1:7" ht="13.5" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="21" spans="1:7" ht="13.5" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="E21" s="1" t="s">
         <v>36</v>
       </c>
@@ -1350,7 +1368,7 @@
         <v>76</v>
       </c>
     </row>
-    <row r="22" spans="1:7" ht="13.5" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="22" spans="1:7" ht="13.5" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="E22" s="1" t="s">
         <v>56</v>
       </c>
@@ -1358,7 +1376,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="23" spans="1:7" ht="13.5" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="23" spans="1:7" ht="13.5" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="E23" s="1" t="s">
         <v>58</v>
       </c>
@@ -1366,7 +1384,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="24" spans="1:7" ht="13.5" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="24" spans="1:7" ht="13.5" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="E24" s="1" t="s">
         <v>60</v>
       </c>
@@ -1374,7 +1392,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="25" spans="1:7" ht="13.5" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="25" spans="1:7" ht="13.5" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="E25" s="1" t="s">
         <v>46</v>
       </c>
@@ -1382,7 +1400,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="26" spans="1:7" ht="13.5" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="26" spans="1:7" ht="13.5" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="E26" s="1" t="s">
         <v>54</v>
       </c>
@@ -1390,7 +1408,7 @@
         <v>82</v>
       </c>
     </row>
-    <row r="27" spans="1:7" ht="13.5" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="27" spans="1:7" ht="13.5" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A27" s="3"/>
       <c r="B27" s="3"/>
       <c r="C27" s="3"/>
@@ -1401,7 +1419,7 @@
       </c>
       <c r="G27" s="3"/>
     </row>
-    <row r="28" spans="1:7" ht="13.5" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="28" spans="1:7" ht="13.5" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A28" s="1" t="s">
         <v>13</v>
       </c>
@@ -1412,42 +1430,42 @@
         <v>40</v>
       </c>
     </row>
-    <row r="29" spans="1:7" ht="13.5" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="29" spans="1:7" ht="13.5" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="C29" s="1" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="30" spans="1:7" ht="13.5" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="30" spans="1:7" ht="13.5" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="C30" s="1" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="31" spans="1:7" ht="13.5" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="31" spans="1:7" ht="13.5" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="C31" s="1" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="32" spans="1:7" ht="13.5" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="32" spans="1:7" ht="13.5" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="C32" s="1" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="33" spans="1:7" ht="13.5" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="33" spans="1:7" ht="13.5" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="C33" s="1" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="34" spans="1:7" ht="13.5" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="34" spans="1:7" ht="13.5" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="C34" s="1" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="35" spans="1:7" ht="13.5" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="35" spans="1:7" ht="13.5" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="C35" s="1" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="36" spans="1:7" ht="13.5" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="36" spans="1:7" ht="13.5" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A36" s="3"/>
       <c r="B36" s="3"/>
       <c r="C36" s="3"/>
@@ -1456,7 +1474,7 @@
       <c r="F36" s="3"/>
       <c r="G36" s="3"/>
     </row>
-    <row r="37" spans="1:7" ht="13.5" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="37" spans="1:7" ht="13.5" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A37" s="1" t="s">
         <v>22</v>
       </c>
@@ -1464,7 +1482,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="38" spans="1:7" ht="13.5" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="38" spans="1:7" ht="13.5" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A38" s="3"/>
       <c r="B38" s="3"/>
       <c r="C38" s="3"/>
@@ -1473,7 +1491,7 @@
       <c r="F38" s="3"/>
       <c r="G38" s="3"/>
     </row>
-    <row r="39" spans="1:7" ht="13.5" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="39" spans="1:7" ht="13.5" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A39" s="1" t="s">
         <v>62</v>
       </c>
@@ -1481,32 +1499,32 @@
         <v>68</v>
       </c>
     </row>
-    <row r="40" spans="1:7" ht="13.5" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="40" spans="1:7" ht="13.5" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="E40" s="1" t="s">
         <v>64</v>
       </c>
     </row>
-    <row r="41" spans="1:7" ht="13.5" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="41" spans="1:7" ht="13.5" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="E41" s="1" t="s">
         <v>65</v>
       </c>
     </row>
-    <row r="42" spans="1:7" ht="13.5" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="42" spans="1:7" ht="13.5" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="E42" s="1" t="s">
         <v>66</v>
       </c>
     </row>
-    <row r="43" spans="1:7" ht="13.5" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="43" spans="1:7" ht="13.5" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="E43" s="1" t="s">
         <v>67</v>
       </c>
     </row>
-    <row r="44" spans="1:7" ht="13.5" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="44" spans="1:7" ht="13.5" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="E44" s="1" t="s">
         <v>63</v>
       </c>
     </row>
-    <row r="45" spans="1:7" ht="13.5" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="45" spans="1:7" ht="13.5" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A45" s="3"/>
       <c r="B45" s="3"/>
       <c r="C45" s="3"/>
@@ -1515,27 +1533,27 @@
       <c r="F45" s="3"/>
       <c r="G45" s="3"/>
     </row>
-    <row r="46" spans="1:7" ht="13.5" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="46" spans="1:7" ht="13.5" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A46" s="1" t="s">
         <v>85</v>
       </c>
     </row>
-    <row r="47" spans="1:7" ht="13.5" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="47" spans="1:7" ht="13.5" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="E47" s="1" t="s">
         <v>87</v>
       </c>
     </row>
-    <row r="48" spans="1:7" ht="13.5" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="48" spans="1:7" ht="13.5" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="E48" s="1" t="s">
         <v>86</v>
       </c>
     </row>
-    <row r="49" spans="1:7" ht="13.5" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="49" spans="1:7" ht="13.5" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="E49" s="1" t="s">
         <v>88</v>
       </c>
     </row>
-    <row r="50" spans="1:7" ht="13.5" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="50" spans="1:7" ht="13.5" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A50" s="3"/>
       <c r="B50" s="3"/>
       <c r="C50" s="3"/>
@@ -1544,12 +1562,12 @@
       <c r="F50" s="3"/>
       <c r="G50" s="3"/>
     </row>
-    <row r="51" spans="1:7" ht="13.5" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="51" spans="1:7" ht="13.5" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A51" s="1" t="s">
         <v>100</v>
       </c>
     </row>
-    <row r="54" spans="1:7" ht="13.5" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="54" spans="1:7" ht="13.5" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A54" s="3"/>
       <c r="B54" s="3"/>
       <c r="C54" s="3"/>
@@ -1558,7 +1576,7 @@
       <c r="F54" s="3"/>
       <c r="G54" s="3"/>
     </row>
-    <row r="55" spans="1:7" ht="13.5" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="55" spans="1:7" ht="13.5" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A55" s="1" t="s">
         <v>24</v>
       </c>
@@ -1578,7 +1596,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="56" spans="1:7" ht="13.5" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="56" spans="1:7" ht="13.5" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A56" s="3"/>
       <c r="B56" s="3"/>
       <c r="C56" s="3"/>
@@ -1602,98 +1620,80 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:G65"/>
-  <sheetFormatPr defaultColWidth="8.69921875" defaultRowHeight="13.5" customHeight="1" x14ac:dyDescent="0.45"/>
+  <dimension ref="A1:G69"/>
+  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="13.5" customHeight="1" x14ac:dyDescent="0.55000000000000004"/>
   <cols>
-    <col min="1" max="1" width="17.19921875" style="1" customWidth="1"/>
-    <col min="2" max="2" width="21.3984375" style="1" customWidth="1"/>
-    <col min="3" max="3" width="29.19921875" style="1" customWidth="1"/>
-    <col min="4" max="4" width="30.09765625" style="1" customWidth="1"/>
-    <col min="5" max="5" width="30.19921875" style="1" customWidth="1"/>
-    <col min="6" max="6" width="26.8984375" style="1" customWidth="1"/>
-    <col min="7" max="7" width="28.796875" style="1" customWidth="1"/>
-    <col min="8" max="16384" width="8.69921875" style="1"/>
+    <col min="1" max="1" width="17.1640625" style="1" customWidth="1"/>
+    <col min="2" max="2" width="21.4140625" style="1" customWidth="1"/>
+    <col min="3" max="3" width="29.1640625" style="1" customWidth="1"/>
+    <col min="4" max="4" width="30.08203125" style="1" customWidth="1"/>
+    <col min="5" max="5" width="30.1640625" style="1" customWidth="1"/>
+    <col min="6" max="6" width="26.9140625" style="1" customWidth="1"/>
+    <col min="7" max="7" width="28.83203125" style="1" customWidth="1"/>
+    <col min="8" max="16384" width="8.6640625" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" ht="31.95" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:7" ht="32" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A1" s="2"/>
       <c r="B1" s="2" t="s">
         <v>101</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>169</v>
+        <v>151</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>170</v>
+        <v>152</v>
       </c>
       <c r="E1" s="2" t="s">
-        <v>171</v>
+        <v>153</v>
       </c>
       <c r="F1" s="2" t="s">
-        <v>172</v>
+        <v>154</v>
       </c>
       <c r="G1" s="2" t="s">
-        <v>173</v>
-      </c>
-    </row>
-    <row r="3" spans="1:7" s="5" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A3" s="5" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" s="4" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+      <c r="A3" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="B3" s="5" t="s">
-        <v>166</v>
-      </c>
-      <c r="C3" s="5" t="s">
-        <v>104</v>
-      </c>
-      <c r="D3" s="5" t="s">
-        <v>106</v>
-      </c>
-      <c r="E3" s="5" t="s">
-        <v>108</v>
-      </c>
-      <c r="F3" s="5" t="s">
-        <v>110</v>
-      </c>
-      <c r="G3" s="5" t="s">
-        <v>112</v>
-      </c>
-    </row>
-    <row r="4" spans="1:7" s="5" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B4" s="5" t="s">
-        <v>167</v>
-      </c>
-      <c r="C4" s="5" t="s">
-        <v>105</v>
-      </c>
-      <c r="D4" s="5" t="s">
-        <v>107</v>
-      </c>
-      <c r="E4" s="5" t="s">
-        <v>109</v>
-      </c>
-      <c r="F4" s="5" t="s">
-        <v>111</v>
-      </c>
-      <c r="G4" s="5" t="s">
-        <v>113</v>
-      </c>
-    </row>
-    <row r="5" spans="1:7" ht="13.5" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="B3" s="4" t="s">
+        <v>157</v>
+      </c>
+      <c r="C3" s="4" t="s">
+        <v>158</v>
+      </c>
+      <c r="D3" s="4" t="s">
+        <v>159</v>
+      </c>
+      <c r="E3" s="4" t="s">
+        <v>160</v>
+      </c>
+      <c r="F3" s="4" t="s">
+        <v>161</v>
+      </c>
+      <c r="G3" s="4" t="s">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" s="4" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.55000000000000004"/>
+    <row r="5" spans="1:7" ht="13.5" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A5" s="3"/>
       <c r="B5" s="3"/>
       <c r="C5" s="3"/>
       <c r="D5" s="3"/>
       <c r="E5" s="3"/>
-      <c r="F5" s="3" t="s">
-        <v>168</v>
-      </c>
+      <c r="F5" s="3"/>
       <c r="G5" s="3"/>
     </row>
-    <row r="6" spans="1:7" ht="13.5" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="6" spans="1:7" ht="13.5" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A6" s="1" t="s">
         <v>6</v>
       </c>
+      <c r="C6" s="1" t="s">
+        <v>7</v>
+      </c>
       <c r="D6" s="1" t="s">
         <v>37</v>
       </c>
@@ -1701,18 +1701,15 @@
         <v>49</v>
       </c>
       <c r="F6" s="1" t="s">
-        <v>132</v>
-      </c>
-      <c r="G6" s="1" t="s">
-        <v>146</v>
-      </c>
-    </row>
-    <row r="7" spans="1:7" ht="13.5" customHeight="1" x14ac:dyDescent="0.45">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" ht="13.5" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A7" s="1" t="s">
         <v>11</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D7" s="1" t="s">
         <v>38</v>
@@ -1721,16 +1718,10 @@
         <v>51</v>
       </c>
       <c r="F7" s="1" t="s">
-        <v>134</v>
-      </c>
-      <c r="G7" s="1" t="s">
-        <v>96</v>
-      </c>
-    </row>
-    <row r="8" spans="1:7" ht="13.5" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="C8" s="1" t="s">
-        <v>8</v>
-      </c>
+        <v>123</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" ht="13.5" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="D8" s="1" t="s">
         <v>32</v>
       </c>
@@ -1738,62 +1729,56 @@
         <v>47</v>
       </c>
       <c r="F8" s="1" t="s">
-        <v>133</v>
-      </c>
-      <c r="G8" s="1" t="s">
-        <v>148</v>
-      </c>
-    </row>
-    <row r="9" spans="1:7" ht="13.5" customHeight="1" x14ac:dyDescent="0.45">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" ht="13.5" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="D9" s="1" t="s">
-        <v>114</v>
+        <v>104</v>
       </c>
       <c r="E9" s="1" t="s">
-        <v>117</v>
+        <v>107</v>
       </c>
       <c r="F9" s="1" t="s">
-        <v>137</v>
-      </c>
-      <c r="G9" s="1" t="s">
-        <v>150</v>
-      </c>
-    </row>
-    <row r="10" spans="1:7" ht="13.5" customHeight="1" x14ac:dyDescent="0.45">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" ht="13.5" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="D10" s="1" t="s">
-        <v>115</v>
+        <v>105</v>
       </c>
       <c r="E10" s="1" t="s">
         <v>61</v>
       </c>
       <c r="F10" s="1" t="s">
-        <v>138</v>
-      </c>
-    </row>
-    <row r="11" spans="1:7" ht="13.5" customHeight="1" x14ac:dyDescent="0.45">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" ht="13.5" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="D11" s="1" t="s">
-        <v>117</v>
+        <v>107</v>
       </c>
       <c r="E11" s="1" t="s">
         <v>35</v>
       </c>
       <c r="F11" s="1" t="s">
-        <v>140</v>
-      </c>
-    </row>
-    <row r="12" spans="1:7" ht="13.5" customHeight="1" x14ac:dyDescent="0.45">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" ht="13.5" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="D12" s="1" t="s">
-        <v>119</v>
+        <v>109</v>
       </c>
       <c r="E12" s="1" t="s">
         <v>55</v>
       </c>
       <c r="F12" s="1" t="s">
-        <v>139</v>
-      </c>
-    </row>
-    <row r="13" spans="1:7" ht="13.5" customHeight="1" x14ac:dyDescent="0.45">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" ht="13.5" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="D13" s="1" t="s">
-        <v>121</v>
+        <v>111</v>
       </c>
       <c r="E13" s="1" t="s">
         <v>57</v>
@@ -1802,441 +1787,479 @@
         <v>79</v>
       </c>
     </row>
-    <row r="14" spans="1:7" ht="13.5" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="14" spans="1:7" ht="13.5" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="D14" s="1" t="s">
-        <v>123</v>
+        <v>113</v>
       </c>
       <c r="E14" s="1" t="s">
         <v>59</v>
       </c>
       <c r="F14" s="1" t="s">
-        <v>131</v>
-      </c>
-    </row>
-    <row r="15" spans="1:7" ht="13.5" customHeight="1" x14ac:dyDescent="0.45">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="15" spans="1:7" ht="13.5" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="D15" s="1" t="s">
-        <v>124</v>
+        <v>114</v>
       </c>
       <c r="E15" s="1" t="s">
         <v>45</v>
       </c>
       <c r="F15" s="1" t="s">
-        <v>143</v>
-      </c>
-    </row>
-    <row r="16" spans="1:7" s="4" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="D16" s="4" t="s">
-        <v>127</v>
+        <v>132</v>
+      </c>
+    </row>
+    <row r="16" spans="1:7" ht="13.5" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+      <c r="D16" s="1" t="s">
+        <v>117</v>
       </c>
       <c r="E16" s="1" t="s">
         <v>53</v>
       </c>
       <c r="F16" s="1" t="s">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6" ht="13.5" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+      <c r="D17" s="1" t="s">
+        <v>61</v>
+      </c>
+      <c r="E17" s="1" t="s">
+        <v>109</v>
+      </c>
+      <c r="F17" s="1" t="s">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6" s="7" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+      <c r="D18" s="7" t="s">
+        <v>118</v>
+      </c>
+      <c r="F18" s="1" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6" s="7" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+      <c r="F19" s="1" t="s">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="20" spans="1:6" s="3" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.55000000000000004"/>
+    <row r="21" spans="1:6" ht="13.5" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+      <c r="A21" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="C21" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="D21" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="E21" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="F21" s="1" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="22" spans="1:6" ht="13.5" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+      <c r="C22" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="D22" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="E22" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="F22" s="1" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="23" spans="1:6" ht="13.5" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+      <c r="D23" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="E23" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="F23" s="1" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="24" spans="1:6" ht="13.5" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+      <c r="D24" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="E24" s="1" t="s">
+        <v>108</v>
+      </c>
+      <c r="F24" s="1" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="25" spans="1:6" ht="13.5" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+      <c r="D25" s="1" t="s">
+        <v>106</v>
+      </c>
+      <c r="E25" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="F25" s="1" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="26" spans="1:6" ht="13.5" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+      <c r="D26" s="1" t="s">
+        <v>108</v>
+      </c>
+      <c r="E26" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="F26" s="1" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="27" spans="1:6" ht="13.5" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+      <c r="D27" s="1" t="s">
+        <v>110</v>
+      </c>
+      <c r="E27" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="F27" s="1" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="28" spans="1:6" ht="13.5" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+      <c r="D28" s="1" t="s">
+        <v>112</v>
+      </c>
+      <c r="E28" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="F28" s="1" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="29" spans="1:6" ht="13.5" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+      <c r="D29" s="1" t="s">
+        <v>115</v>
+      </c>
+      <c r="E29" s="1" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="30" spans="1:6" ht="13.5" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+      <c r="D30" s="1" t="s">
+        <v>116</v>
+      </c>
+      <c r="E30" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="F30" s="1" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="31" spans="1:6" ht="13.5" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+      <c r="D31" s="1" t="s">
+        <v>117</v>
+      </c>
+      <c r="E31" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="F31" s="1" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="32" spans="1:6" ht="13.5" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+      <c r="D32" s="1" t="s">
+        <v>61</v>
+      </c>
+      <c r="E32" s="1" t="s">
+        <v>110</v>
+      </c>
+      <c r="F32" s="1" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="33" spans="1:7" s="7" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+      <c r="D33" s="7" t="s">
+        <v>118</v>
+      </c>
+      <c r="F33" s="1" t="s">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="34" spans="1:7" s="7" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+      <c r="F34" s="1" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="35" spans="1:7" s="3" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.55000000000000004"/>
+    <row r="36" spans="1:7" ht="13.5" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+      <c r="A36" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="C36" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="D36" s="1" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="37" spans="1:7" ht="13.5" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+      <c r="C37" s="1" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="38" spans="1:7" ht="13.5" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+      <c r="C38" s="1" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="39" spans="1:7" ht="13.5" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+      <c r="C39" s="1" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="40" spans="1:7" ht="13.5" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+      <c r="C40" s="1" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="41" spans="1:7" ht="13.5" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+      <c r="C41" s="1" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="42" spans="1:7" ht="13.5" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+      <c r="C42" s="1" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="43" spans="1:7" ht="13.5" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+      <c r="C43" s="1" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="44" spans="1:7" ht="13.5" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+      <c r="A44" s="3"/>
+      <c r="B44" s="3"/>
+      <c r="C44" s="3"/>
+      <c r="D44" s="3"/>
+      <c r="E44" s="3"/>
+      <c r="F44" s="3"/>
+      <c r="G44" s="3"/>
+    </row>
+    <row r="45" spans="1:7" ht="13.5" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+      <c r="A45" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="B45" s="5" t="s">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="46" spans="1:7" ht="13.5" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+      <c r="A46" s="3"/>
+      <c r="B46" s="6"/>
+      <c r="C46" s="3"/>
+      <c r="D46" s="3"/>
+      <c r="E46" s="3"/>
+      <c r="F46" s="3"/>
+      <c r="G46" s="3"/>
+    </row>
+    <row r="47" spans="1:7" ht="13.5" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+      <c r="A47" s="1" t="s">
+        <v>163</v>
+      </c>
+      <c r="C47" s="1" t="s">
+        <v>137</v>
+      </c>
+      <c r="E47" s="1" t="s">
+        <v>119</v>
+      </c>
+      <c r="F47" s="1" t="s">
+        <v>134</v>
+      </c>
+      <c r="G47" s="1" t="s">
         <v>142</v>
       </c>
     </row>
-    <row r="17" spans="1:7" ht="13.5" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A17" s="4"/>
-      <c r="B17" s="4"/>
-      <c r="C17" s="4"/>
-      <c r="D17" s="4" t="s">
-        <v>61</v>
-      </c>
-      <c r="E17" s="1" t="s">
-        <v>119</v>
-      </c>
-      <c r="F17" s="4"/>
-      <c r="G17" s="4"/>
-    </row>
-    <row r="18" spans="1:7" s="3" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="D18" s="3" t="s">
-        <v>128</v>
-      </c>
-    </row>
-    <row r="19" spans="1:7" ht="13.5" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A19" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="C19" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="D19" s="1" t="s">
-        <v>39</v>
-      </c>
-      <c r="E19" s="1" t="s">
-        <v>50</v>
-      </c>
-      <c r="F19" s="1" t="s">
-        <v>83</v>
-      </c>
-      <c r="G19" s="1" t="s">
+    <row r="48" spans="1:7" ht="13.5" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+      <c r="C48" s="1" t="s">
+        <v>138</v>
+      </c>
+      <c r="E48" s="1" t="s">
+        <v>140</v>
+      </c>
+      <c r="F48" s="1" t="s">
+        <v>141</v>
+      </c>
+      <c r="G48" s="1" t="s">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="49" spans="1:7" ht="13.5" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+      <c r="C49" s="1" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="50" spans="1:7" ht="13.5" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+      <c r="A50" s="3"/>
+      <c r="B50" s="3"/>
+      <c r="C50" s="3"/>
+      <c r="D50" s="3"/>
+      <c r="E50" s="3"/>
+      <c r="F50" s="3"/>
+      <c r="G50" s="3"/>
+    </row>
+    <row r="51" spans="1:7" ht="13.5" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+      <c r="A51" s="7" t="s">
+        <v>165</v>
+      </c>
+      <c r="B51" s="7"/>
+      <c r="C51" s="8" t="s">
+        <v>166</v>
+      </c>
+      <c r="D51" s="7"/>
+      <c r="E51" s="7"/>
+      <c r="F51" s="7"/>
+      <c r="G51" s="7" t="s">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="52" spans="1:7" ht="13.5" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+      <c r="A52" s="7"/>
+      <c r="B52" s="7"/>
+      <c r="C52" s="8" t="s">
+        <v>167</v>
+      </c>
+      <c r="D52" s="7"/>
+      <c r="E52" s="7"/>
+      <c r="F52" s="7"/>
+      <c r="G52" s="7" t="s">
+        <v>171</v>
+      </c>
+    </row>
+    <row r="53" spans="1:7" ht="13.5" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+      <c r="A53" s="7"/>
+      <c r="B53" s="7"/>
+      <c r="C53" s="7"/>
+      <c r="D53" s="7"/>
+      <c r="E53" s="7"/>
+      <c r="F53" s="7"/>
+      <c r="G53" s="7" t="s">
+        <v>172</v>
+      </c>
+    </row>
+    <row r="54" spans="1:7" ht="13.5" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+      <c r="A54" s="7"/>
+      <c r="B54" s="7"/>
+      <c r="C54" s="7"/>
+      <c r="D54" s="7"/>
+      <c r="E54" s="7"/>
+      <c r="F54" s="7"/>
+      <c r="G54" s="7" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="55" spans="1:7" ht="13.5" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+      <c r="A55" s="7"/>
+      <c r="B55" s="7"/>
+      <c r="C55" s="7"/>
+      <c r="D55" s="7"/>
+      <c r="E55" s="7"/>
+      <c r="F55" s="7"/>
+      <c r="G55" s="7" t="s">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="56" spans="1:7" ht="13.5" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+      <c r="A56" s="7"/>
+      <c r="B56" s="7"/>
+      <c r="C56" s="7"/>
+      <c r="D56" s="7"/>
+      <c r="E56" s="7"/>
+      <c r="F56" s="7"/>
+      <c r="G56" s="7"/>
+    </row>
+    <row r="57" spans="1:7" s="3" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.55000000000000004"/>
+    <row r="58" spans="1:7" ht="13.5" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+      <c r="A58" s="1" t="s">
+        <v>164</v>
+      </c>
+      <c r="F58" s="2" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="59" spans="1:7" ht="13.5" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+      <c r="F59" s="2" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="60" spans="1:7" ht="13.5" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+      <c r="F60" s="2" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="61" spans="1:7" ht="13.5" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+      <c r="F61" s="2" t="s">
         <v>147</v>
       </c>
     </row>
-    <row r="20" spans="1:7" ht="13.5" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="C20" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="D20" s="1" t="s">
-        <v>29</v>
-      </c>
-      <c r="E20" s="1" t="s">
-        <v>52</v>
-      </c>
-      <c r="F20" s="1" t="s">
-        <v>135</v>
-      </c>
-      <c r="G20" s="1" t="s">
-        <v>97</v>
-      </c>
-    </row>
-    <row r="21" spans="1:7" ht="13.5" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="D21" s="1" t="s">
-        <v>33</v>
-      </c>
-      <c r="E21" s="1" t="s">
-        <v>48</v>
-      </c>
-      <c r="F21" s="1" t="s">
-        <v>136</v>
-      </c>
-      <c r="G21" s="1" t="s">
+    <row r="62" spans="1:7" ht="13.5" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+      <c r="F62" s="2" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="63" spans="1:7" ht="13.5" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+      <c r="F63" s="2" t="s">
         <v>149</v>
       </c>
     </row>
-    <row r="22" spans="1:7" ht="13.5" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="D22" s="1" t="s">
-        <v>31</v>
-      </c>
-      <c r="E22" s="1" t="s">
-        <v>118</v>
-      </c>
-      <c r="F22" s="1" t="s">
-        <v>81</v>
-      </c>
-      <c r="G22" s="1" t="s">
-        <v>151</v>
-      </c>
-    </row>
-    <row r="23" spans="1:7" ht="13.5" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="D23" s="1" t="s">
-        <v>116</v>
-      </c>
-      <c r="E23" s="1" t="s">
-        <v>34</v>
-      </c>
-      <c r="F23" s="1" t="s">
-        <v>82</v>
-      </c>
-    </row>
-    <row r="24" spans="1:7" ht="13.5" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="D24" s="1" t="s">
-        <v>118</v>
-      </c>
-      <c r="E24" s="1" t="s">
-        <v>36</v>
-      </c>
-      <c r="F24" s="1" t="s">
-        <v>76</v>
-      </c>
-    </row>
-    <row r="25" spans="1:7" ht="13.5" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="D25" s="1" t="s">
-        <v>120</v>
-      </c>
-      <c r="E25" s="1" t="s">
-        <v>56</v>
-      </c>
-      <c r="F25" s="1" t="s">
-        <v>79</v>
-      </c>
-    </row>
-    <row r="26" spans="1:7" ht="13.5" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="D26" s="1" t="s">
-        <v>122</v>
-      </c>
-      <c r="E26" s="1" t="s">
-        <v>58</v>
-      </c>
-      <c r="F26" s="1" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="27" spans="1:7" ht="13.5" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="D27" s="1" t="s">
-        <v>125</v>
-      </c>
-      <c r="E27" s="1" t="s">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="28" spans="1:7" ht="13.5" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="D28" s="1" t="s">
-        <v>126</v>
-      </c>
-      <c r="E28" s="1" t="s">
-        <v>46</v>
-      </c>
-      <c r="F28" s="4" t="s">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="29" spans="1:7" s="4" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="D29" s="4" t="s">
-        <v>127</v>
-      </c>
-      <c r="E29" s="1" t="s">
-        <v>54</v>
-      </c>
-      <c r="F29" s="1" t="s">
-        <v>144</v>
-      </c>
-    </row>
-    <row r="30" spans="1:7" ht="13.5" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A30" s="4"/>
-      <c r="B30" s="4"/>
-      <c r="C30" s="4"/>
-      <c r="D30" s="4" t="s">
-        <v>61</v>
-      </c>
-      <c r="E30" s="1" t="s">
-        <v>120</v>
-      </c>
-      <c r="F30" s="1" t="s">
-        <v>141</v>
-      </c>
-      <c r="G30" s="4"/>
-    </row>
-    <row r="31" spans="1:7" s="3" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="D31" s="3" t="s">
-        <v>128</v>
-      </c>
-    </row>
-    <row r="32" spans="1:7" ht="13.5" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A32" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="C32" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="D32" s="1" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="33" spans="1:7" ht="13.5" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="C33" s="1" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="34" spans="1:7" ht="13.5" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="C34" s="1" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="35" spans="1:7" ht="13.5" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="C35" s="1" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="36" spans="1:7" ht="13.5" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="C36" s="1" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="37" spans="1:7" ht="13.5" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="C37" s="1" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="38" spans="1:7" ht="13.5" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="C38" s="1" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="39" spans="1:7" ht="13.5" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="C39" s="1" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="40" spans="1:7" ht="13.5" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A40" s="3"/>
-      <c r="B40" s="3"/>
-      <c r="C40" s="3"/>
-      <c r="D40" s="3"/>
-      <c r="E40" s="3"/>
-      <c r="F40" s="3"/>
-      <c r="G40" s="3"/>
-    </row>
-    <row r="41" spans="1:7" ht="13.5" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A41" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="B41" s="6" t="s">
-        <v>174</v>
-      </c>
-    </row>
-    <row r="42" spans="1:7" ht="13.5" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A42" s="3"/>
-      <c r="B42" s="7"/>
-      <c r="C42" s="3"/>
-      <c r="D42" s="3"/>
-      <c r="E42" s="3"/>
-      <c r="F42" s="3"/>
-      <c r="G42" s="3"/>
-    </row>
-    <row r="43" spans="1:7" ht="13.5" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A43" s="1" t="s">
-        <v>62</v>
-      </c>
-      <c r="E43" s="1" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="44" spans="1:7" ht="13.5" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="E44" s="1" t="s">
-        <v>64</v>
-      </c>
-    </row>
-    <row r="45" spans="1:7" ht="13.5" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="E45" s="1" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="46" spans="1:7" ht="13.5" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="E46" s="1" t="s">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="47" spans="1:7" ht="13.5" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="E47" s="1" t="s">
-        <v>67</v>
-      </c>
-    </row>
-    <row r="49" spans="1:7" ht="13.5" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A49" s="3"/>
-      <c r="B49" s="3"/>
-      <c r="C49" s="3"/>
-      <c r="D49" s="3"/>
-      <c r="E49" s="3"/>
-      <c r="F49" s="3"/>
-      <c r="G49" s="3"/>
-    </row>
-    <row r="50" spans="1:7" ht="13.5" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A50" s="1" t="s">
-        <v>85</v>
-      </c>
-    </row>
-    <row r="51" spans="1:7" ht="13.5" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="E51" s="1" t="s">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="52" spans="1:7" ht="13.5" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="E52" s="1" t="s">
-        <v>88</v>
-      </c>
-    </row>
-    <row r="54" spans="1:7" ht="13.5" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A54" s="3"/>
-      <c r="B54" s="3"/>
-      <c r="C54" s="3"/>
-      <c r="D54" s="3"/>
-      <c r="E54" s="3"/>
-      <c r="F54" s="3"/>
-      <c r="G54" s="3"/>
-    </row>
-    <row r="55" spans="1:7" ht="13.5" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A55" s="1" t="s">
-        <v>100</v>
-      </c>
-      <c r="C55" s="1" t="s">
-        <v>152</v>
-      </c>
-      <c r="E55" s="1" t="s">
-        <v>129</v>
-      </c>
-      <c r="F55" s="1" t="s">
-        <v>145</v>
-      </c>
-      <c r="G55" s="1" t="s">
-        <v>157</v>
-      </c>
-    </row>
-    <row r="56" spans="1:7" ht="13.5" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="C56" s="1" t="s">
-        <v>153</v>
-      </c>
-      <c r="E56" s="1" t="s">
-        <v>155</v>
-      </c>
-      <c r="F56" s="1" t="s">
-        <v>156</v>
-      </c>
-      <c r="G56" s="1" t="s">
-        <v>158</v>
-      </c>
-    </row>
-    <row r="57" spans="1:7" ht="13.5" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="C57" s="1" t="s">
-        <v>154</v>
-      </c>
-    </row>
-    <row r="58" spans="1:7" ht="13.5" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A58" s="3"/>
-      <c r="B58" s="3"/>
-      <c r="C58" s="3"/>
-      <c r="D58" s="3"/>
-      <c r="E58" s="3"/>
-      <c r="F58" s="3"/>
-      <c r="G58" s="3"/>
-    </row>
-    <row r="59" spans="1:7" ht="13.5" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A59" s="1" t="s">
-        <v>130</v>
-      </c>
-      <c r="F59" s="1" t="s">
-        <v>159</v>
-      </c>
-    </row>
-    <row r="60" spans="1:7" ht="13.5" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="F60" s="1" t="s">
-        <v>160</v>
-      </c>
-    </row>
-    <row r="61" spans="1:7" ht="13.5" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="F61" s="1" t="s">
-        <v>161</v>
-      </c>
-    </row>
-    <row r="62" spans="1:7" ht="13.5" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="F62" s="1" t="s">
-        <v>162</v>
-      </c>
-    </row>
-    <row r="63" spans="1:7" ht="13.5" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="F63" s="1" t="s">
-        <v>163</v>
-      </c>
-    </row>
-    <row r="64" spans="1:7" ht="13.5" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="F64" s="1" t="s">
-        <v>164</v>
-      </c>
-    </row>
-    <row r="65" spans="1:7" ht="13.5" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A65" s="3"/>
-      <c r="B65" s="3"/>
-      <c r="C65" s="3"/>
-      <c r="D65" s="3"/>
-      <c r="E65" s="3"/>
-      <c r="F65" s="3" t="s">
-        <v>165</v>
-      </c>
-      <c r="G65" s="3"/>
+    <row r="64" spans="1:7" ht="13.5" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+      <c r="A64" s="3"/>
+      <c r="B64" s="3"/>
+      <c r="C64" s="3"/>
+      <c r="D64" s="3"/>
+      <c r="E64" s="3"/>
+      <c r="F64" s="9" t="s">
+        <v>150</v>
+      </c>
+      <c r="G64" s="3"/>
+    </row>
+    <row r="65" spans="1:7" ht="13.5" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+      <c r="A65" s="1" t="s">
+        <v>175</v>
+      </c>
+      <c r="G65" s="1" t="s">
+        <v>176</v>
+      </c>
+    </row>
+    <row r="66" spans="1:7" ht="13.5" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+      <c r="G66" s="1" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="67" spans="1:7" ht="13.5" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+      <c r="G67" s="1" t="s">
+        <v>178</v>
+      </c>
+    </row>
+    <row r="68" spans="1:7" ht="13.5" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+      <c r="G68" s="1" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="69" spans="1:7" s="3" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+      <c r="G69" s="3" t="s">
+        <v>180</v>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="B41:B42"/>
+    <mergeCell ref="B45:B46"/>
   </mergeCells>
   <phoneticPr fontId="1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>